<commit_message>
2026-10-23 weekly: 주간보고 현황 갱신
</commit_message>
<xml_diff>
--- a/_attic/docs/개발현황.xlsx
+++ b/_attic/docs/개발현황.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2182건 (회사 기간 670건)</t>
+          <t>2208건 (회사 기간 670건)</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>112 / 121개 (93%)</t>
+          <t>113 / 122개 (93%)</t>
         </is>
       </c>
     </row>
@@ -4590,14 +4590,14 @@
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t>■</t>
+            <t>■■■■■■■■■■■■■</t>
           </r>
           <r>
             <rPr>
               <color rgb="00000000"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">  (1)</t>
+            <t xml:space="preserve">  (27)</t>
           </r>
         </is>
       </c>
@@ -5382,7 +5382,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" ht="113.4" customHeight="1">
+    <row r="26" ht="162" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>2026-10-19 ~ 10-23</t>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>불량·관리·작업 예약 개선</t>
+          <t>불량·예약·실사·출하 개선</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -5401,11 +5401,14 @@
 품목 검색과 입출고 내역 확인 편의 개선
 컴퓨터·모바일 입출고 방향 안내와 취소 처리 개선
 작업 예약·공유 작업 현황 및 상세 확인 추가
-전수조사 대기 화면과 로그인 로고 표시 개선</t>
+전수조사 중 기존 작업 보존·예약 해제와 조사 반영 후 이어하기
+출하 작업자 입력과 전체 작업 확인 통합
+부족 자재의 확보 가능 수량 예약과 제출 제한 보완 진행 중
+로그인 로고 표시 개선</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>91</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -5419,7 +5422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8173,27 +8176,27 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="12" t="n">
+      <c r="A114" s="9" t="n">
         <v>113</v>
       </c>
-      <c r="B114" s="13" t="inlineStr">
-        <is>
-          <t>실 재고 데이터 입력 + 직원 테스트</t>
-        </is>
-      </c>
-      <c r="C114" s="12" t="inlineStr">
-        <is>
-          <t>데이터</t>
-        </is>
-      </c>
-      <c r="D114" s="14" t="inlineStr">
-        <is>
-          <t>🔲 예정</t>
-        </is>
-      </c>
-      <c r="E114" s="13" t="inlineStr">
-        <is>
-          <t>BOM·입출고 정리 후</t>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>전수조사 중 작업 일시중지·재개</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>재고</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="inlineStr">
+        <is>
+          <t>기존 작업·수량을 보존하고 예약 해제 후 조사 반영 시 이어하기</t>
         </is>
       </c>
     </row>
@@ -8203,12 +8206,12 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>불량 처리 흐름 Phase 2</t>
+          <t>실 재고 데이터 입력 + 직원 테스트</t>
         </is>
       </c>
       <c r="C115" s="12" t="inlineStr">
         <is>
-          <t>생산</t>
+          <t>데이터</t>
         </is>
       </c>
       <c r="D115" s="14" t="inlineStr">
@@ -8218,7 +8221,7 @@
       </c>
       <c r="E115" s="13" t="inlineStr">
         <is>
-          <t>부서 결재·집계·자동화</t>
+          <t>BOM·입출고 정리 후</t>
         </is>
       </c>
     </row>
@@ -8228,12 +8231,12 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>역할별 접근 권한 연동</t>
+          <t>불량 처리 흐름 Phase 2</t>
         </is>
       </c>
       <c r="C116" s="12" t="inlineStr">
         <is>
-          <t>보안</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="D116" s="14" t="inlineStr">
@@ -8243,7 +8246,7 @@
       </c>
       <c r="E116" s="13" t="inlineStr">
         <is>
-          <t>부서·역할 기반 (PIN 로그인 완료)</t>
+          <t>부서 결재·집계·자동화</t>
         </is>
       </c>
     </row>
@@ -8253,12 +8256,12 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>총재고 / 가용재고 / 예약재고 분리</t>
+          <t>역할별 접근 권한 연동</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr">
         <is>
-          <t>재고</t>
+          <t>보안</t>
         </is>
       </c>
       <c r="D117" s="14" t="inlineStr">
@@ -8268,7 +8271,7 @@
       </c>
       <c r="E117" s="13" t="inlineStr">
         <is>
-          <t>재고 가용성 계산 고도화</t>
+          <t>부서·역할 기반 (PIN 로그인 완료)</t>
         </is>
       </c>
     </row>
@@ -8278,12 +8281,12 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>외부 접근 환경 구성</t>
+          <t>총재고 / 가용재고 / 예약재고 분리</t>
         </is>
       </c>
       <c r="C118" s="12" t="inlineStr">
         <is>
-          <t>인프라</t>
+          <t>재고</t>
         </is>
       </c>
       <c r="D118" s="14" t="inlineStr">
@@ -8293,7 +8296,7 @@
       </c>
       <c r="E118" s="13" t="inlineStr">
         <is>
-          <t>PC 또는 NAS 서버 + API 인증</t>
+          <t>재고 가용성 계산 고도화</t>
         </is>
       </c>
     </row>
@@ -8303,12 +8306,12 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>발주 관리</t>
+          <t>외부 접근 환경 구성</t>
         </is>
       </c>
       <c r="C119" s="12" t="inlineStr">
         <is>
-          <t>구매</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
@@ -8316,7 +8319,11 @@
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E119" s="13" t="inlineStr"/>
+      <c r="E119" s="13" t="inlineStr">
+        <is>
+          <t>PC 또는 NAS 서버 + API 인증</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="n">
@@ -8324,12 +8331,12 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>생산 실적 / 원가 관리</t>
+          <t>발주 관리</t>
         </is>
       </c>
       <c r="C120" s="12" t="inlineStr">
         <is>
-          <t>생산</t>
+          <t>구매</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
@@ -8345,12 +8352,12 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>부서별 생산진행도 대시보드</t>
+          <t>생산 실적 / 원가 관리</t>
         </is>
       </c>
       <c r="C121" s="12" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
@@ -8358,11 +8365,7 @@
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E121" s="13" t="inlineStr">
-        <is>
-          <t>사장님 요청 — 검토 중</t>
-        </is>
-      </c>
+      <c r="E121" s="13" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="12" t="n">
@@ -8370,20 +8373,45 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
+          <t>부서별 생산진행도 대시보드</t>
+        </is>
+      </c>
+      <c r="C122" s="12" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D122" s="14" t="inlineStr">
+        <is>
+          <t>🔲 예정</t>
+        </is>
+      </c>
+      <c r="E122" s="13" t="inlineStr">
+        <is>
+          <t>사장님 요청 — 검토 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="12" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
           <t>출하 거래처 관리</t>
         </is>
       </c>
-      <c r="C122" s="12" t="inlineStr">
+      <c r="C123" s="12" t="inlineStr">
         <is>
           <t>출하</t>
         </is>
       </c>
-      <c r="D122" s="14" t="inlineStr">
+      <c r="D123" s="14" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E122" s="13" t="inlineStr">
+      <c r="E123" s="13" t="inlineStr">
         <is>
           <t>거래처 마스터 + 출하 이력</t>
         </is>
@@ -11609,18 +11637,22 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="27" customHeight="1">
+    <row r="136" ht="67.5" customHeight="1">
       <c r="A136" s="15" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
       <c r="B136" s="15" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="C136" s="16" t="inlineStr">
         <is>
-          <t>2026-10-23 frontend: 대시보드 스켈레톤 스크롤 높이를 실제 목록과 동기화</t>
+          <t>2026-10-23 frontend: 대시보드 스켈레톤 스크롤 높이를 실제 목록과 동기화
+2026-10-23 frontend: 일보 불량 재작업 상세 표시 수정
+2026-10-23 frontend: 일보 상세 펼침 시 작업 내역 높이 유지
+2026-10-23 backend: 재제출 이전 취소 이력을 승인 완료 집계에서 제외
+2026-10-23 backend: 과거 일부 완료 작업의 안전한 상태 정정 도구 추가</t>
         </is>
       </c>
       <c r="D136" s="15" t="inlineStr">
@@ -11640,7 +11672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2183"/>
+  <dimension ref="A1:F2209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -81507,6 +81539,838 @@
         </is>
       </c>
     </row>
+    <row r="2184">
+      <c r="A2184" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2184" s="15" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C2184" s="15" t="inlineStr">
+        <is>
+          <t>e9a4374e</t>
+        </is>
+      </c>
+      <c r="D2184" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 일보 불량 재작업 상세 표시 수정</t>
+        </is>
+      </c>
+      <c r="E2184" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2184" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2185" s="7" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="C2185" s="7" t="inlineStr">
+        <is>
+          <t>adc33780</t>
+        </is>
+      </c>
+      <c r="D2185" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 일보 상세 펼침 시 작업 내역 높이 유지</t>
+        </is>
+      </c>
+      <c r="E2185" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2185" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2186" s="15" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C2186" s="15" t="inlineStr">
+        <is>
+          <t>33f862f0</t>
+        </is>
+      </c>
+      <c r="D2186" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 backend: 재제출 이전 취소 이력을 승인 완료 집계에서 제외</t>
+        </is>
+      </c>
+      <c r="E2186" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F2186" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2187" s="7" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C2187" s="7" t="inlineStr">
+        <is>
+          <t>26d7f1e6</t>
+        </is>
+      </c>
+      <c r="D2187" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 backend: 과거 일부 완료 작업의 안전한 상태 정정 도구 추가</t>
+        </is>
+      </c>
+      <c r="E2187" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F2187" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2188" s="15" t="inlineStr">
+        <is>
+          <t>09:36</t>
+        </is>
+      </c>
+      <c r="C2188" s="15" t="inlineStr">
+        <is>
+          <t>c7fe0dc1</t>
+        </is>
+      </c>
+      <c r="D2188" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 대시보드와 상세 수량 갱신 동기화</t>
+        </is>
+      </c>
+      <c r="E2188" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2188" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2189" s="7" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C2189" s="7" t="inlineStr">
+        <is>
+          <t>0dcffb88</t>
+        </is>
+      </c>
+      <c r="D2189" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 로그인 로고 로딩과 모바일 배치 개선</t>
+        </is>
+      </c>
+      <c r="E2189" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2189" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2190" s="15" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C2190" s="15" t="inlineStr">
+        <is>
+          <t>b5a7b852</t>
+        </is>
+      </c>
+      <c r="D2190" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 docs: 주간보고와 개발현황을 10월 23일 기준으로 갱신</t>
+        </is>
+      </c>
+      <c r="E2190" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F2190" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2191" s="7" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C2191" s="7" t="inlineStr">
+        <is>
+          <t>f1f72c15</t>
+        </is>
+      </c>
+      <c r="D2191" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 docs: 메인과 병합 후보 비교 검증 계획 추가</t>
+        </is>
+      </c>
+      <c r="E2191" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F2191" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2192" s="15" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C2192" s="15" t="inlineStr">
+        <is>
+          <t>9a76c769</t>
+        </is>
+      </c>
+      <c r="D2192" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 전체 작업 기본 정렬을 부서순으로 변경</t>
+        </is>
+      </c>
+      <c r="E2192" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2192" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2193" s="7" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C2193" s="7" t="inlineStr">
+        <is>
+          <t>29a849ec</t>
+        </is>
+      </c>
+      <c r="D2193" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 입출고 메모 공유와 작업 목록 표시 정리</t>
+        </is>
+      </c>
+      <c r="E2193" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2193" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2194" s="15" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C2194" s="15" t="inlineStr">
+        <is>
+          <t>3359b3a7</t>
+        </is>
+      </c>
+      <c r="D2194" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 부서 결재 담당자의 전체 작업 기본 진입 적용</t>
+        </is>
+      </c>
+      <c r="E2194" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2194" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2195" s="7" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C2195" s="7" t="inlineStr">
+        <is>
+          <t>56853ed9</t>
+        </is>
+      </c>
+      <c r="D2195" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 예정 변동 배지를 한 줄로 통일</t>
+        </is>
+      </c>
+      <c r="E2195" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2195" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2196" s="15" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C2196" s="15" t="inlineStr">
+        <is>
+          <t>b10b3d69</t>
+        </is>
+      </c>
+      <c r="D2196" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 backend: 저장 작업 건수와 단건 조회 및 일괄 읽기 최적화</t>
+        </is>
+      </c>
+      <c r="E2196" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F2196" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2197" s="7" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C2197" s="7" t="inlineStr">
+        <is>
+          <t>ae0007d1</t>
+        </is>
+      </c>
+      <c r="D2197" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 로그인 경계의 작업 캐시와 조회 정책 정리</t>
+        </is>
+      </c>
+      <c r="E2197" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2197" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2198" s="15" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C2198" s="15" t="inlineStr">
+        <is>
+          <t>674274dd</t>
+        </is>
+      </c>
+      <c r="D2198" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 작업 건수 분리와 최신 저장 작업 복원 적용</t>
+        </is>
+      </c>
+      <c r="E2198" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2198" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2199" s="7" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C2199" s="7" t="inlineStr">
+        <is>
+          <t>03570757</t>
+        </is>
+      </c>
+      <c r="D2199" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 backend: 전수조사 작업 일시중지 모델과 마이그레이션 추가</t>
+        </is>
+      </c>
+      <c r="E2199" s="7" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F2199" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2200" s="15" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C2200" s="15" t="inlineStr">
+        <is>
+          <t>706019b4</t>
+        </is>
+      </c>
+      <c r="D2200" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 backend: 전수조사 작업 예약 해제와 원자적 재개 구현</t>
+        </is>
+      </c>
+      <c r="E2200" s="15" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F2200" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2201" s="7" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C2201" s="7" t="inlineStr">
+        <is>
+          <t>d9278105</t>
+        </is>
+      </c>
+      <c r="D2201" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 일시중지 상태와 예약 관리 이력 표시</t>
+        </is>
+      </c>
+      <c r="E2201" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2201" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2202" s="15" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C2202" s="15" t="inlineStr">
+        <is>
+          <t>58748514</t>
+        </is>
+      </c>
+      <c r="D2202" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 조사 반영 후 기존 수량으로 바로 작업 이어가기</t>
+        </is>
+      </c>
+      <c r="E2202" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2202" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2203" s="7" t="inlineStr">
+        <is>
+          <t>12:16</t>
+        </is>
+      </c>
+      <c r="C2203" s="7" t="inlineStr">
+        <is>
+          <t>8efb0464</t>
+        </is>
+      </c>
+      <c r="D2203" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 docs: 작업 일시중지 재개 정책과 검증 기록 정리</t>
+        </is>
+      </c>
+      <c r="E2203" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F2203" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2204" s="15" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C2204" s="15" t="inlineStr">
+        <is>
+          <t>7b990e43</t>
+        </is>
+      </c>
+      <c r="D2204" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 튜닝 직원의 입출고 품목 전환 허용</t>
+        </is>
+      </c>
+      <c r="E2204" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2204" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2205" s="7" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C2205" s="7" t="inlineStr">
+        <is>
+          <t>b1e85d8e</t>
+        </is>
+      </c>
+      <c r="D2205" s="8" t="inlineStr">
+        <is>
+          <t>Merge commit '8efb04648e0b9f2b795b2d0c149c2537bb9498d2' into HEAD</t>
+        </is>
+      </c>
+      <c r="E2205" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2205" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2206" s="15" t="inlineStr">
+        <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="C2206" s="15" t="inlineStr">
+        <is>
+          <t>6f9966e9</t>
+        </is>
+      </c>
+      <c r="D2206" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 warehouse: 튜닝 직원 품목 전환 허용 롤백</t>
+        </is>
+      </c>
+      <c r="E2206" s="15" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2206" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2207" s="7" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C2207" s="7" t="inlineStr">
+        <is>
+          <t>a28b4335</t>
+        </is>
+      </c>
+      <c r="D2207" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 shipping: 출하 작업자 입력과 전체 작업 통합</t>
+        </is>
+      </c>
+      <c r="E2207" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2207" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2208" s="15" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C2208" s="15" t="inlineStr">
+        <is>
+          <t>89752e5b</t>
+        </is>
+      </c>
+      <c r="D2208" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-23 frontend: 출하 상세 진입 로딩과 요약 중앙 정렬 개선</t>
+        </is>
+      </c>
+      <c r="E2208" s="15" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F2208" s="15" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2209" s="7" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C2209" s="7" t="inlineStr">
+        <is>
+          <t>5f62956b</t>
+        </is>
+      </c>
+      <c r="D2209" s="8" t="inlineStr">
+        <is>
+          <t>Merge branch 'main' into HEAD</t>
+        </is>
+      </c>
+      <c r="E2209" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F2209" s="7" t="inlineStr">
+        <is>
+          <t>근무</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>